<commit_message>
Day 5 — Added slicers, conditional formatting and dashboard polish
</commit_message>
<xml_diff>
--- a/Sales_Dashboard_Project.xlsx
+++ b/Sales_Dashboard_Project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cb05eb62caaf167c/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="373" documentId="8_{E7AF8C15-64D3-4F33-84D9-7927CA658BA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8B7D9D72-11B3-4856-BF8E-DD0747E7E107}"/>
+  <xr:revisionPtr revIDLastSave="453" documentId="8_{E7AF8C15-64D3-4F33-84D9-7927CA658BA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0552ED3C-92B1-4954-A488-CB6218EF6F45}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{3FCCABB5-28AF-4571-AA11-A83FDF695285}"/>
   </bookViews>
@@ -17,11 +17,26 @@
     <sheet name="ANALYSIS" sheetId="3" r:id="rId2"/>
     <sheet name="DASHBOARD" sheetId="5" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="Slicer_Category">#N/A</definedName>
+    <definedName name="Slicer_Region">#N/A</definedName>
+    <definedName name="Slicer_Salesperson">#N/A</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="8" r:id="rId4"/>
+    <pivotCache cacheId="0" r:id="rId4"/>
   </pivotCaches>
   <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
+      <x14:slicerCaches>
+        <x14:slicerCache r:id="rId5"/>
+        <x14:slicerCache r:id="rId6"/>
+        <x14:slicerCache r:id="rId7"/>
+      </x14:slicerCaches>
+    </ext>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
+      <x14:workbookPr/>
+    </ext>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
@@ -198,7 +213,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -206,31 +221,90 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top style="thick">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
+      </left>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top style="thick">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thick">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <numFmt numFmtId="22" formatCode="mmm/yy"/>
     </dxf>
@@ -1337,6 +1411,7 @@
           </a:p>
         </c:txPr>
         <c:crossAx val="1109819711"/>
+        <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -1395,6 +1470,7 @@
           </a:p>
         </c:txPr>
         <c:crossAx val="1109807711"/>
+        <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:spPr>
@@ -2077,6 +2153,7 @@
           </a:p>
         </c:txPr>
         <c:crossAx val="1109827871"/>
+        <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -2135,6 +2212,7 @@
           </a:p>
         </c:txPr>
         <c:crossAx val="1109825951"/>
+        <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:spPr>
@@ -4028,7 +4106,245 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>23049</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>27064</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>921225</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>22745</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="5" name="Category">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ECC911B2-8147-E716-19DD-2931F2079EA4}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2010/slicer">
+              <sle:slicer xmlns:sle="http://schemas.microsoft.com/office/drawing/2010/slicer" name="Category"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="1330959" y="4098646"/>
+              <a:ext cx="2160594" cy="3089174"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-IN" sz="1100"/>
+                <a:t>This shape represents a slicer. Slicers are supported in Excel 2010 or later.
+If the shape was modified in an earlier version of Excel, or if the workbook was saved in Excel 2003 or earlier, the slicer cannot be used.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>3525</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>20358</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>604026</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>54051</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="8" name="Region">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F45794A6-5BE8-7762-D758-42E88AF11BCE}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2010/slicer">
+              <sle:slicer xmlns:sle="http://schemas.microsoft.com/office/drawing/2010/slicer" name="Region"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="6383853" y="4091940"/>
+              <a:ext cx="1828800" cy="2581275"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-IN" sz="1100"/>
+                <a:t>This shape represents a slicer. Slicers are supported in Excel 2010 or later.
+If the shape was modified in an earlier version of Excel, or if the workbook was saved in Excel 2003 or earlier, the slicer cannot be used.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>14900</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>43104</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>1252</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>76797</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="9" name="Salesperson">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{936C7AAB-CD57-B49E-8BF1-CD7FAD05AC2A}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2010/slicer">
+              <sle:slicer xmlns:sle="http://schemas.microsoft.com/office/drawing/2010/slicer" name="Salesperson"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="10694273" y="4114686"/>
+              <a:ext cx="1828800" cy="2581275"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-IN" sz="1100"/>
+                <a:t>This shape represents a slicer. Slicers are supported in Excel 2010 or later.
+If the shape was modified in an earlier version of Excel, or if the workbook was saved in Excel 2003 or earlier, the slicer cannot be used.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4080,7 +4396,7 @@
   </cacheFields>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
-      <x14:pivotCacheDefinition/>
+      <x14:pivotCacheDefinition pivotCacheId="1925419808"/>
     </ext>
   </extLst>
 </pivotCacheDefinition>
@@ -4312,7 +4628,110 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0C565B64-9909-4127-BB10-493782562243}" name="PivotTable4" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E56E0921-3CA6-466F-AB73-55EFD059A592}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
+  <location ref="A1:B4" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="9">
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="17" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="5">
+        <item x="2"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="5">
+        <item x="2"/>
+        <item x="1"/>
+        <item x="0"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="3"/>
+  </rowFields>
+  <rowItems count="3">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of Total Sales" fld="8" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="3">
+    <chartFormat chart="2" format="4" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="2" format="5">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="3" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="2" format="6">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="3" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0C565B64-9909-4127-BB10-493782562243}" name="PivotTable4" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
   <location ref="K1:L6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField showAll="0"/>
@@ -4430,8 +4849,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9904B653-ED69-4219-9A23-A49321FE3FF4}" name="PivotTable3" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6">
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9904B653-ED69-4219-9A23-A49321FE3FF4}" name="PivotTable3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6">
   <location ref="F1:G6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField showAll="0"/>
@@ -4549,91 +4968,64 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E56E0921-3CA6-466F-AB73-55EFD059A592}" name="PivotTable1" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
-  <location ref="A1:B4" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="9">
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="17" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="3">
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
+<file path=xl/slicerCaches/slicerCache1.xml><?xml version="1.0" encoding="utf-8"?>
+<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_Category" xr10:uid="{6711E09B-080A-4F4A-BC0D-06449E33EC09}" sourceName="Category">
+  <pivotTables>
+    <pivotTable tabId="3" name="PivotTable1"/>
+  </pivotTables>
+  <data>
+    <tabular pivotCacheId="1925419808">
+      <items count="2">
+        <i x="0" s="1"/>
+        <i x="1" s="1"/>
       </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="3"/>
-  </rowFields>
-  <rowItems count="3">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Sum of Total Sales" fld="8" baseField="0" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="3">
-    <chartFormat chart="2" format="4" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="2" format="5">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="3" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="2" format="6">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="3" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
+    </tabular>
+  </data>
+</slicerCacheDefinition>
+</file>
+
+<file path=xl/slicerCaches/slicerCache2.xml><?xml version="1.0" encoding="utf-8"?>
+<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_Region" xr10:uid="{DCEED614-72E7-4987-AECF-BB1F286E0942}" sourceName="Region">
+  <pivotTables>
+    <pivotTable tabId="3" name="PivotTable3"/>
+  </pivotTables>
+  <data>
+    <tabular pivotCacheId="1925419808">
+      <items count="4">
+        <i x="2" s="1"/>
+        <i x="0" s="1"/>
+        <i x="1" s="1"/>
+        <i x="3" s="1"/>
+      </items>
+    </tabular>
+  </data>
+</slicerCacheDefinition>
+</file>
+
+<file path=xl/slicerCaches/slicerCache3.xml><?xml version="1.0" encoding="utf-8"?>
+<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_Salesperson" xr10:uid="{AAAAA4EA-A8E9-4B9B-8821-072CCBDBB78B}" sourceName="Salesperson">
+  <pivotTables>
+    <pivotTable tabId="3" name="PivotTable4"/>
+  </pivotTables>
+  <data>
+    <tabular pivotCacheId="1925419808">
+      <items count="4">
+        <i x="2" s="1"/>
+        <i x="1" s="1"/>
+        <i x="0" s="1"/>
+        <i x="3" s="1"/>
+      </items>
+    </tabular>
+  </data>
+</slicerCacheDefinition>
+</file>
+
+<file path=xl/slicers/slicer1.xml><?xml version="1.0" encoding="utf-8"?>
+<slicers xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10">
+  <slicer name="Category" xr10:uid="{536F5D5E-5D35-4DE8-A30C-1A0DFAE9C582}" cache="Slicer_Category" caption="Filter By Category" rowHeight="247650"/>
+  <slicer name="Region" xr10:uid="{7DEDD243-2518-4DFE-8048-003CFE9CF924}" cache="Slicer_Region" caption="Filter By Region" rowHeight="247650"/>
+  <slicer name="Salesperson" xr10:uid="{1D8ECDB6-E531-448C-BF2C-CA46D3C133D4}" cache="Slicer_Salesperson" caption="Filter By Salesperson" rowHeight="247650"/>
+</slicers>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4641,7 +5033,7 @@
   <autoFilter ref="A1:I21" xr:uid="{A8472A96-FA4B-4191-8811-7629704B6A93}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{FE638889-D6FA-47BC-B9D2-28496D625645}" name="Order ID"/>
-    <tableColumn id="2" xr3:uid="{411CCF91-F79E-42EF-A4E7-FE8E66234F31}" name="Date" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{411CCF91-F79E-42EF-A4E7-FE8E66234F31}" name="Date" dataDxfId="1"/>
     <tableColumn id="3" xr3:uid="{D4CF904B-DD3D-4AB8-A52D-FC4E7A33894B}" name="Product"/>
     <tableColumn id="4" xr3:uid="{6EA4D58B-54D3-44E9-B9F6-9691352DE4B0}" name="Category"/>
     <tableColumn id="5" xr3:uid="{CB91FFC4-E4C2-4951-9194-5093F81D3D6D}" name="Region"/>
@@ -5660,19 +6052,19 @@
       <c r="A2" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="4">
+      <c r="B2" s="6">
         <v>2311000</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="G2" s="4">
+      <c r="G2" s="6">
         <v>631500</v>
       </c>
       <c r="K2" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="L2" s="4">
+      <c r="L2" s="6">
         <v>631500</v>
       </c>
     </row>
@@ -5680,19 +6072,19 @@
       <c r="A3" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="4">
+      <c r="B3" s="6">
         <v>440000</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="G3" s="4">
+      <c r="G3" s="6">
         <v>707500</v>
       </c>
       <c r="K3" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="L3" s="4">
+      <c r="L3" s="6">
         <v>912000</v>
       </c>
     </row>
@@ -5700,19 +6092,19 @@
       <c r="A4" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="6">
         <v>2751000</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="G4" s="4">
+      <c r="G4" s="6">
         <v>912000</v>
       </c>
       <c r="K4" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="L4" s="4">
+      <c r="L4" s="6">
         <v>707500</v>
       </c>
     </row>
@@ -5720,13 +6112,13 @@
       <c r="F5" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="G5" s="4">
+      <c r="G5" s="6">
         <v>500000</v>
       </c>
       <c r="K5" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="L5" s="4">
+      <c r="L5" s="6">
         <v>500000</v>
       </c>
     </row>
@@ -5734,13 +6126,13 @@
       <c r="F6" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="G6" s="4">
+      <c r="G6" s="6">
         <v>2751000</v>
       </c>
       <c r="K6" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="L6" s="4">
+      <c r="L6" s="6">
         <v>2751000</v>
       </c>
     </row>
@@ -5751,17 +6143,17 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C887CFE-6E3E-4889-B422-B936D2CB7BBB}">
-  <dimension ref="A1:S3"/>
+  <dimension ref="A1:S4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:19" ht="24" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="4" t="s">
         <v>29</v>
       </c>
       <c r="B1" s="5"/>
@@ -5783,39 +6175,55 @@
       <c r="R1" s="5"/>
       <c r="S1" s="5"/>
     </row>
-    <row r="2" spans="1:19" ht="18" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:19" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="9" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:19" ht="18" x14ac:dyDescent="0.35">
-      <c r="A3" s="8">
+    <row r="3" spans="1:19" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="10">
         <v>2751000</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="9" t="s">
         <v>23</v>
       </c>
     </row>
+    <row r="4" spans="1:19" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:S1"/>
   </mergeCells>
+  <conditionalFormatting sqref="A3">
+    <cfRule type="cellIs" priority="2" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{A8765BA9-456A-4dab-B4F3-ACF838C121DE}">
+      <x14:slicerList>
+        <x14:slicer r:id="rId2"/>
+      </x14:slicerList>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
</xml_diff>